<commit_message>
Actualizacion de datos financieros en Excel
</commit_message>
<xml_diff>
--- a/Datos/Gestion Proyecto Fatima.xlsx
+++ b/Datos/Gestion Proyecto Fatima.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP I5\Documents\Dashboard_Obras\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434582C6-B063-4A49-AD3C-3E1E14C5AA28}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C281F4E4-604E-4624-A9BC-3B8106A5AD0A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1522,13 +1522,13 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -5078,14 +5078,12 @@
     <sheetNames>
       <sheetName val="Panel_de_Control"/>
       <sheetName val="Registro_Transacciones"/>
-      <sheetName val="Soporte de compras"/>
       <sheetName val="Configuracion"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -5498,7 +5496,7 @@
       </c>
       <c r="C2" s="69">
         <f>[1]!Panel_Control[[#This Row],[Total Ejecutado]]</f>
-        <v>25621.65</v>
+        <v>28026.52</v>
       </c>
       <c r="D2" s="68">
         <f>[1]!Panel_Control[[#This Row],[Total Ingresos]]</f>
@@ -5506,7 +5504,7 @@
       </c>
       <c r="E2" s="68">
         <f t="shared" ref="E2:E8" si="0">D2-C2</f>
-        <v>8153.5</v>
+        <v>5748.630000000001</v>
       </c>
       <c r="F2" s="68">
         <f t="shared" ref="F2:G4" si="1">B2-D2</f>
@@ -5514,15 +5512,15 @@
       </c>
       <c r="G2" s="68">
         <f t="shared" si="1"/>
-        <v>17468.150000000001</v>
+        <v>22277.89</v>
       </c>
       <c r="H2" s="68">
         <f t="shared" ref="H2:H8" si="2">E2</f>
-        <v>8153.5</v>
+        <v>5748.630000000001</v>
       </c>
       <c r="I2" s="72">
         <f t="shared" ref="I2:I8" si="3">C2/B2</f>
-        <v>0.66367324926656146</v>
+        <v>0.72596618851768979</v>
       </c>
       <c r="J2" s="72">
         <f t="shared" ref="J2:J8" si="4">D2/B2</f>
@@ -5530,7 +5528,7 @@
       </c>
       <c r="K2" s="68">
         <f t="shared" ref="K2:K8" si="5">B2-C2</f>
-        <v>12984.169999999998</v>
+        <v>10579.3</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -5813,7 +5811,7 @@
       </c>
       <c r="C9" s="73">
         <f>SUM(C2:C8)</f>
-        <v>29451.65</v>
+        <v>31856.52</v>
       </c>
       <c r="D9" s="73">
         <f>SUM(D2:D8)</f>
@@ -5821,7 +5819,7 @@
       </c>
       <c r="E9" s="68">
         <f t="shared" ref="E9" si="8">D9-C9</f>
-        <v>23812.25</v>
+        <v>21407.38</v>
       </c>
       <c r="F9" s="68">
         <f t="shared" ref="F9" si="9">B9-D9</f>
@@ -5829,15 +5827,15 @@
       </c>
       <c r="G9" s="68">
         <f t="shared" ref="G9" si="10">C9-E9</f>
-        <v>5639.4000000000015</v>
+        <v>10449.14</v>
       </c>
       <c r="H9" s="68">
         <f t="shared" ref="H9" si="11">E9</f>
-        <v>23812.25</v>
+        <v>21407.38</v>
       </c>
       <c r="I9" s="72">
         <f t="shared" ref="I9" si="12">C9/B9</f>
-        <v>0.44594414941941174</v>
+        <v>0.48235765109467477</v>
       </c>
       <c r="J9" s="72">
         <f t="shared" ref="J9" si="13">D9/B9</f>
@@ -5845,7 +5843,7 @@
       </c>
       <c r="K9" s="68">
         <f t="shared" ref="K9" si="14">B9-C9</f>
-        <v>36591.71</v>
+        <v>34186.839999999997</v>
       </c>
     </row>
   </sheetData>
@@ -5870,28 +5868,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="77" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="79"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="74" t="s">
@@ -5927,7 +5925,7 @@
         <v>22037.563618134853</v>
       </c>
       <c r="F5" s="75"/>
-      <c r="G5" s="77">
+      <c r="G5" s="79">
         <f>C5/A5</f>
         <v>0.49710716525496096</v>
       </c>
@@ -5977,7 +5975,7 @@
         <v>11419.963618134854</v>
       </c>
       <c r="F8" s="75"/>
-      <c r="G8" s="77">
+      <c r="G8" s="79">
         <f>C8/A8</f>
         <v>0.65606652639833785</v>
       </c>
@@ -6211,6 +6209,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:D9"/>
+    <mergeCell ref="E8:F9"/>
+    <mergeCell ref="G8:H9"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
@@ -6220,14 +6226,6 @@
     <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H6"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:D9"/>
-    <mergeCell ref="E8:F9"/>
-    <mergeCell ref="G8:H9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -6247,20 +6245,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="79"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -6402,32 +6400,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="79"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -10875,38 +10873,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="77" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="79"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">

</xml_diff>